<commit_message>
Penambahan fitur check out
</commit_message>
<xml_diff>
--- a/SIT_Report.xlsx
+++ b/SIT_Report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -35,7 +35,7 @@
     <t>SUCCESS</t>
   </si>
   <si>
-    <t>2026-03-25 02:11:14</t>
+    <t>2026-03-29 20:40:06</t>
   </si>
   <si>
     <t>SIT-002</t>
@@ -44,10 +44,34 @@
     <t>Add To Cart</t>
   </si>
   <si>
+    <t>2026-03-29 20:40:09</t>
+  </si>
+  <si>
     <t>SIT-003</t>
   </si>
   <si>
     <t>Remove Item</t>
+  </si>
+  <si>
+    <t>2026-03-29 20:40:12</t>
+  </si>
+  <si>
+    <t>SIT-004</t>
+  </si>
+  <si>
+    <t>Checkout Positive</t>
+  </si>
+  <si>
+    <t>2026-03-29 20:40:37</t>
+  </si>
+  <si>
+    <t>SIT-005</t>
+  </si>
+  <si>
+    <t>Checkout Negative</t>
+  </si>
+  <si>
+    <t>2026-03-29 20:40:52</t>
   </si>
 </sst>
 </file>
@@ -92,7 +116,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -134,21 +158,49 @@
         <v>6</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s" s="0">
         <v>6</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>7</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added TestNG validation on test folder and testng xml on root folder
</commit_message>
<xml_diff>
--- a/SIT_Report.xlsx
+++ b/SIT_Report.xlsx
@@ -35,7 +35,7 @@
     <t>SUCCESS</t>
   </si>
   <si>
-    <t>2026-03-29 20:40:06</t>
+    <t>2026-03-30 22:25:31</t>
   </si>
   <si>
     <t>SIT-002</t>
@@ -44,7 +44,7 @@
     <t>Add To Cart</t>
   </si>
   <si>
-    <t>2026-03-29 20:40:09</t>
+    <t>2026-03-30 22:25:33</t>
   </si>
   <si>
     <t>SIT-003</t>
@@ -53,16 +53,16 @@
     <t>Remove Item</t>
   </si>
   <si>
-    <t>2026-03-29 20:40:12</t>
+    <t>2026-03-30 22:25:35</t>
   </si>
   <si>
     <t>SIT-004</t>
   </si>
   <si>
-    <t>Checkout Positive</t>
-  </si>
-  <si>
-    <t>2026-03-29 20:40:37</t>
+    <t>Checkout</t>
+  </si>
+  <si>
+    <t>2026-03-30 22:25:52</t>
   </si>
   <si>
     <t>SIT-005</t>
@@ -71,7 +71,7 @@
     <t>Checkout Negative</t>
   </si>
   <si>
-    <t>2026-03-29 20:40:52</t>
+    <t>2026-03-30 22:26:02</t>
   </si>
 </sst>
 </file>

</xml_diff>